<commit_message>
Switch RENOVIT packaging model to 25kg bags
</commit_message>
<xml_diff>
--- a/data/technology/RENOVIT_Technology_CAPEX_Model.xlsx
+++ b/data/technology/RENOVIT_Technology_CAPEX_Model.xlsx
@@ -551,7 +551,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>30kg bagging machine</t>
+          <t>25kg bagging machine</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -566,7 +566,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>30kg filled bags</t>
+          <t>25kg filled bags</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -870,7 +870,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>30kg bagging line</t>
+          <t>25kg bagging line</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">

</xml_diff>

<commit_message>
Correct limestone process map and visual assets
</commit_message>
<xml_diff>
--- a/data/technology/RENOVIT_Technology_CAPEX_Model.xlsx
+++ b/data/technology/RENOVIT_Technology_CAPEX_Model.xlsx
@@ -1924,7 +1924,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Limestone and bentonite selection</t>
+          <t>Selective quarrying and sample coding</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1944,12 +1944,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Selected feedstock</t>
+          <t>Coded and separated feedstock</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Which zones provide the best whiteness / volume / bentonite activity?</t>
+          <t>Which zones give best whiteness and stability for the premium line?</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -1959,7 +1959,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Take coded samples by source and zone</t>
+          <t>White material must stay physically separated from bulk material</t>
         </is>
       </c>
     </row>
@@ -1989,7 +1989,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Limestone at Ocnita plant</t>
+          <t>White limestone at Ocnita plant</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -2014,12 +2014,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Pre-crushing / feed preparation</t>
+          <t>Pre-crushing and metal separation</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Crusher or existing preparation line</t>
+          <t>Crusher + magnet + aspiration</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -2034,22 +2034,22 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Prepared feed for milling</t>
+          <t>Prepared feed for further processing</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Can Ocnita flour residue be used directly for adhesive?</t>
+          <t>Can Ocnita flour residue be used directly in adhesive after QC?</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>working_assumption</t>
+          <t>critical</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Depends on purity and contamination of residue</t>
+          <t>Protects fine grinding equipment and product cleanliness</t>
         </is>
       </c>
     </row>
@@ -2059,12 +2059,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Micronization</t>
+          <t>Conditional drying / moisture conditioning</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Micronizer / fine mill</t>
+          <t>Dryer or covered conditioning stock</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -2074,27 +2074,27 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Prepared limestone</t>
+          <t>Prepared feed</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Extra-fine calcium carbonate filler</t>
+          <t>Feed within target moisture</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>What fineness is required for glet extra-white?</t>
+          <t>Do we need drying at all or can covered stock do the job?</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>critical</t>
+          <t>working_assumption</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Replaces gypsum calcination as main quality bottleneck</t>
+          <t>Dry only if moisture breaks process spec</t>
         </is>
       </c>
     </row>
@@ -2104,12 +2104,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Granulometric sorting</t>
+          <t>Route A ultrafine grinding</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Sieves / classifier</t>
+          <t>Micronizer / fine mill</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -2119,17 +2119,17 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Ground limestone</t>
+          <t>Prepared white limestone</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Controlled fractions</t>
+          <t>Ultrafine calcium carbonate filler</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>What fractions are needed for decorative render?</t>
+          <t>What fineness is required for glet extra-white?</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -2139,7 +2139,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Controls texture and repeatability</t>
+          <t>Main quality bottleneck for premium skim coat</t>
         </is>
       </c>
     </row>
@@ -2149,32 +2149,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Additive dosing</t>
+          <t>Route B coarse screening for decorative fractions</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Dosing units</t>
+          <t>Sieves / crusher / classifier</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2-8 percent of mix</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Limestone filler + additives</t>
+          <t>Prepared limestone</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Dosed blend</t>
+          <t>Controlled decorative fractions</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Which additives are needed for each recipe?</t>
+          <t>What aggregate cuts are needed for decorative render?</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -2184,7 +2184,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Polymers cellulose lime/cement may drive cost</t>
+          <t>Decorative fractions should not be modeled as fully micronized powder</t>
         </is>
       </c>
     </row>
@@ -2194,32 +2194,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Dry mixing</t>
+          <t>Binder and additive dosing</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Industrial dry mixer</t>
+          <t>Dosing units for cement / lime / cellulose / RDP</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>around 10 t/hour</t>
+          <t>2-12 percent of mix</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
+          <t>Filler / fractions + binder system</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
           <t>Dosed blend</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Homogeneous dry mix</t>
-        </is>
-      </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Can mixer keep recipe consistency?</t>
+          <t>Which binder system is correct for each SKU?</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -2229,7 +2229,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Homogeneity affects claims and returns</t>
+          <t>Filler alone is not enough; each product family needs its own binder system</t>
         </is>
       </c>
     </row>
@@ -2239,32 +2239,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Quality control</t>
+          <t>Campaign dry mixing</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Lab equipment</t>
+          <t>Industrial dry mixer</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>around 10 t/hour</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Lot samples</t>
+          <t>Dosed blend</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Approved / rejected lot</t>
+          <t>Homogeneous dry mix</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Which tests are done per batch?</t>
+          <t>Can one or two mixers support SKU campaigns in phase 1?</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -2274,7 +2274,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Whiteness granulometry adhesion setting time</t>
+          <t>More realistic than three dedicated lines at launch</t>
         </is>
       </c>
     </row>
@@ -2284,12 +2284,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Bulk / product storage</t>
+          <t>Product-specific quality control</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Silo / big bags</t>
+          <t>Lab equipment</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -2299,27 +2299,27 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Approved dry mix</t>
+          <t>Lot samples</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Stored product</t>
+          <t>Approved / rejected lot</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>How much buffer stock is needed?</t>
+          <t>Which tests are required for EN 998-1 and EN 12004 routes?</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>working_assumption</t>
+          <t>critical</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Moisture control is key</t>
+          <t>Check whiteness PSD moisture workability adhesion and permeability</t>
         </is>
       </c>
     </row>
@@ -2329,42 +2329,42 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Bag filling</t>
+          <t>Bulk storage and release silos</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Adjustable 20/25kg bagging machine</t>
+          <t>Silo / big bags</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>600 bags/hour</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Bulk product</t>
+          <t>Approved dry mix</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Filled bags</t>
+          <t>Released product</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Can line handle both 20kg and 25kg formats?</t>
+          <t>How much protected buffer stock is needed?</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>critical</t>
+          <t>working_assumption</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Commercial bottleneck for retail-ready product</t>
+          <t>Moisture control and white-line cleanliness are critical</t>
         </is>
       </c>
     </row>
@@ -2374,42 +2374,42 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Stitching and printing</t>
+          <t>Bag filling</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Bag stitcher + printer</t>
+          <t>Adjustable 20/25kg bagging machine</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>500-800 bags/hour</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
+          <t>Bulk product</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
           <t>Filled bags</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Sealed labelled bags</t>
-        </is>
-      </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>What label / compliance information is required?</t>
+          <t>Can one flexible line cover launch volumes?</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>critical</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Connects quality and product readiness</t>
+          <t>One strong flexible line is more realistic than three packers at launch</t>
         </is>
       </c>
     </row>
@@ -2419,7 +2419,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Palletizing</t>
+          <t>Palletizing and dry warehouse</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2434,7 +2434,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Sealed bags</t>
+          <t>Filled bags</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -2444,7 +2444,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Manual now or robot later?</t>
+          <t>What stock age and FIFO policy do we need?</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -2454,7 +2454,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Robot likely not needed in phase 1</t>
+          <t>Needs dry warehouse and clean changeover discipline</t>
         </is>
       </c>
     </row>
@@ -2464,12 +2464,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Finished goods storage and loading</t>
+          <t>Loading and dispatch</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Forklift + warehouse</t>
+          <t>Forklift + warehouse + road or rail</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -2489,7 +2489,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>How many days of finished goods stock are needed?</t>
+          <t>What mix of road and rail actually makes sense from Ocnita?</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -2499,7 +2499,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Needs dry warehouse and moisture control</t>
+          <t>Logistics node matters but does not change chemistry of the process</t>
         </is>
       </c>
     </row>

</xml_diff>